<commit_message>
Add pre-split data, evaluation protocol and pseudo-code starter
- data/: CoverType (covtype.csv.gz) and split_metadata.csv (train/eval, stratified, seed 42)
- scripts/: split_data.py, evaluate.py (accuracy, macro-F1, per-class, confusion matrix), make_split_metadata.py
- code/: pseudo-code skeleton (data, model, optimizer, train, plots, results_table, lab.ipynb)
- RUBRIC: eval score section (15 points), thresholds on eval macro-F1
- README/GUIDE/REPORT_TEMPLATE/xlsx updated for train/eval protocol and submission list

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/experiment_table_template.xlsx
+++ b/templates/experiment_table_template.xlsx
@@ -280,19 +280,19 @@
     <t xml:space="preserve">Loss thành NaN/inf? Y | N</t>
   </si>
   <si>
-    <t xml:space="preserve">test_acc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test accuracy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHỈ điền cho baseline và cấu hình cuối cùng.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_macro_f1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test macro-F1</t>
+    <t xml:space="preserve">eval_acc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accuracy trên tập eval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHỈ điền cho baseline và cấu hình cuối cùng, lấy từ eval_result.json.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eval_macro_f1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">macro-F1 trên tập eval</t>
   </si>
   <si>
     <t xml:space="preserve">figure_file</t>
@@ -1350,7 +1350,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
         <v>84</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
         <v>87</v>
       </c>

</xml_diff>